<commit_message>
UK daily ratings for 2026-05-30
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-05-30.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-05-30.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P276"/>
+  <dimension ref="A1:P332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -882,14 +882,14 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Cornish Pol (IRE)</t>
+          <t>Rollthedicebaby (IRE)</t>
         </is>
       </c>
       <c r="I8" t="n">
         <v>2</v>
       </c>
       <c r="J8" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -938,14 +938,14 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Rollthedicebaby (IRE)</t>
+          <t>Cornish Pol (IRE)</t>
         </is>
       </c>
       <c r="I9" t="n">
         <v>2</v>
       </c>
       <c r="J9" t="n">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -3140,17 +3140,17 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Nakatomi (IRE)</t>
+          <t>Langton Wold (IRE)</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J46" t="n">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="K46" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="n">
@@ -3196,17 +3196,17 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Langton Wold (IRE)</t>
+          <t>Nakatomi (IRE)</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J47" t="n">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="K47" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="n">
@@ -16842,6 +16842,3336 @@
       </c>
       <c r="P276" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>1</v>
+      </c>
+      <c r="C277" t="n">
+        <v>11.60454545454546</v>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F277" t="n">
+        <v>6</v>
+      </c>
+      <c r="G277" t="n">
+        <v>0</v>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>Mick The Hat (IRE)</t>
+        </is>
+      </c>
+      <c r="I277" t="n">
+        <v>3</v>
+      </c>
+      <c r="J277" t="n">
+        <v>135</v>
+      </c>
+      <c r="K277" t="n">
+        <v>55</v>
+      </c>
+      <c r="L277" t="inlineStr"/>
+      <c r="M277" t="n">
+        <v>149.53</v>
+      </c>
+      <c r="N277" t="inlineStr"/>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P277" t="n">
+        <v>-11.5</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>1</v>
+      </c>
+      <c r="C278" t="n">
+        <v>11.60454545454546</v>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F278" t="n">
+        <v>6</v>
+      </c>
+      <c r="G278" t="n">
+        <v>0</v>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>Panthere Noir</t>
+        </is>
+      </c>
+      <c r="I278" t="n">
+        <v>3</v>
+      </c>
+      <c r="J278" t="n">
+        <v>129</v>
+      </c>
+      <c r="K278" t="n">
+        <v>49</v>
+      </c>
+      <c r="L278" t="inlineStr"/>
+      <c r="M278" t="n">
+        <v>149.53</v>
+      </c>
+      <c r="N278" t="inlineStr"/>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P278" t="n">
+        <v>-11.5</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>1</v>
+      </c>
+      <c r="C279" t="n">
+        <v>11.60454545454546</v>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F279" t="n">
+        <v>6</v>
+      </c>
+      <c r="G279" t="n">
+        <v>1</v>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Song Of The Stars</t>
+        </is>
+      </c>
+      <c r="I279" t="n">
+        <v>3</v>
+      </c>
+      <c r="J279" t="n">
+        <v>133</v>
+      </c>
+      <c r="K279" t="n">
+        <v>53</v>
+      </c>
+      <c r="L279" t="inlineStr"/>
+      <c r="M279" t="n">
+        <v>149.53</v>
+      </c>
+      <c r="N279" t="n">
+        <v>74.7</v>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P279" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>1</v>
+      </c>
+      <c r="C280" t="n">
+        <v>11.60454545454546</v>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F280" t="n">
+        <v>6</v>
+      </c>
+      <c r="G280" t="n">
+        <v>2</v>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>Naranka (IRE)</t>
+        </is>
+      </c>
+      <c r="I280" t="n">
+        <v>3</v>
+      </c>
+      <c r="J280" t="n">
+        <v>126</v>
+      </c>
+      <c r="K280" t="n">
+        <v>46</v>
+      </c>
+      <c r="L280" t="n">
+        <v>2</v>
+      </c>
+      <c r="M280" t="n">
+        <v>149.53</v>
+      </c>
+      <c r="N280" t="n">
+        <v>68</v>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P280" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>1</v>
+      </c>
+      <c r="C281" t="n">
+        <v>11.60454545454546</v>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F281" t="n">
+        <v>6</v>
+      </c>
+      <c r="G281" t="n">
+        <v>3</v>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Head Girl</t>
+        </is>
+      </c>
+      <c r="I281" t="n">
+        <v>3</v>
+      </c>
+      <c r="J281" t="n">
+        <v>132</v>
+      </c>
+      <c r="K281" t="n">
+        <v>52</v>
+      </c>
+      <c r="L281" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="M281" t="n">
+        <v>149.53</v>
+      </c>
+      <c r="N281" t="n">
+        <v>70.59999999999999</v>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P281" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>1</v>
+      </c>
+      <c r="C282" t="n">
+        <v>11.60454545454546</v>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F282" t="n">
+        <v>6</v>
+      </c>
+      <c r="G282" t="n">
+        <v>4</v>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Timely Salute</t>
+        </is>
+      </c>
+      <c r="I282" t="n">
+        <v>3</v>
+      </c>
+      <c r="J282" t="n">
+        <v>132</v>
+      </c>
+      <c r="K282" t="n">
+        <v>52</v>
+      </c>
+      <c r="L282" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="M282" t="n">
+        <v>149.53</v>
+      </c>
+      <c r="N282" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P282" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>1</v>
+      </c>
+      <c r="C283" t="n">
+        <v>11.60454545454546</v>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F283" t="n">
+        <v>6</v>
+      </c>
+      <c r="G283" t="n">
+        <v>5</v>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Lucky Sevens</t>
+        </is>
+      </c>
+      <c r="I283" t="n">
+        <v>3</v>
+      </c>
+      <c r="J283" t="n">
+        <v>135</v>
+      </c>
+      <c r="K283" t="n">
+        <v>55</v>
+      </c>
+      <c r="L283" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="M283" t="n">
+        <v>149.53</v>
+      </c>
+      <c r="N283" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P283" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>1</v>
+      </c>
+      <c r="C284" t="n">
+        <v>11.60454545454546</v>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F284" t="n">
+        <v>6</v>
+      </c>
+      <c r="G284" t="n">
+        <v>6</v>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Keep It Classic</t>
+        </is>
+      </c>
+      <c r="I284" t="n">
+        <v>3</v>
+      </c>
+      <c r="J284" t="n">
+        <v>133</v>
+      </c>
+      <c r="K284" t="n">
+        <v>53</v>
+      </c>
+      <c r="L284" t="n">
+        <v>13.45</v>
+      </c>
+      <c r="M284" t="n">
+        <v>149.53</v>
+      </c>
+      <c r="N284" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P284" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>1</v>
+      </c>
+      <c r="C285" t="n">
+        <v>11.60454545454546</v>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F285" t="n">
+        <v>6</v>
+      </c>
+      <c r="G285" t="n">
+        <v>7</v>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Fletcher</t>
+        </is>
+      </c>
+      <c r="I285" t="n">
+        <v>3</v>
+      </c>
+      <c r="J285" t="n">
+        <v>131</v>
+      </c>
+      <c r="K285" t="n">
+        <v>51</v>
+      </c>
+      <c r="L285" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="M285" t="n">
+        <v>149.53</v>
+      </c>
+      <c r="N285" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P285" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>1</v>
+      </c>
+      <c r="C286" t="n">
+        <v>11.60454545454546</v>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F286" t="n">
+        <v>6</v>
+      </c>
+      <c r="G286" t="n">
+        <v>8</v>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Mister Pretentious</t>
+        </is>
+      </c>
+      <c r="I286" t="n">
+        <v>3</v>
+      </c>
+      <c r="J286" t="n">
+        <v>126</v>
+      </c>
+      <c r="K286" t="n">
+        <v>46</v>
+      </c>
+      <c r="L286" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="M286" t="n">
+        <v>149.53</v>
+      </c>
+      <c r="N286" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P286" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>1</v>
+      </c>
+      <c r="C287" t="n">
+        <v>11.60454545454546</v>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F287" t="n">
+        <v>6</v>
+      </c>
+      <c r="G287" t="n">
+        <v>9</v>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Ada Rose</t>
+        </is>
+      </c>
+      <c r="I287" t="n">
+        <v>3</v>
+      </c>
+      <c r="J287" t="n">
+        <v>132</v>
+      </c>
+      <c r="K287" t="n">
+        <v>52</v>
+      </c>
+      <c r="L287" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="M287" t="n">
+        <v>149.53</v>
+      </c>
+      <c r="N287" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P287" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>1</v>
+      </c>
+      <c r="C288" t="n">
+        <v>11.60454545454546</v>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F288" t="n">
+        <v>6</v>
+      </c>
+      <c r="G288" t="n">
+        <v>10</v>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Out In The Cold (IRE)</t>
+        </is>
+      </c>
+      <c r="I288" t="n">
+        <v>3</v>
+      </c>
+      <c r="J288" t="n">
+        <v>126</v>
+      </c>
+      <c r="K288" t="n">
+        <v>46</v>
+      </c>
+      <c r="L288" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="M288" t="n">
+        <v>149.53</v>
+      </c>
+      <c r="N288" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P288" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>2</v>
+      </c>
+      <c r="C289" t="n">
+        <v>10</v>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F289" t="n">
+        <v>6</v>
+      </c>
+      <c r="G289" t="n">
+        <v>1</v>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Pride Of Nepal</t>
+        </is>
+      </c>
+      <c r="I289" t="n">
+        <v>8</v>
+      </c>
+      <c r="J289" t="n">
+        <v>137</v>
+      </c>
+      <c r="K289" t="n">
+        <v>57</v>
+      </c>
+      <c r="L289" t="inlineStr"/>
+      <c r="M289" t="n">
+        <v>127.66</v>
+      </c>
+      <c r="N289" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P289" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>2</v>
+      </c>
+      <c r="C290" t="n">
+        <v>10</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F290" t="n">
+        <v>6</v>
+      </c>
+      <c r="G290" t="n">
+        <v>2</v>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Shifra (IRE)</t>
+        </is>
+      </c>
+      <c r="I290" t="n">
+        <v>4</v>
+      </c>
+      <c r="J290" t="n">
+        <v>126</v>
+      </c>
+      <c r="K290" t="n">
+        <v>46</v>
+      </c>
+      <c r="L290" t="n">
+        <v>1</v>
+      </c>
+      <c r="M290" t="n">
+        <v>127.66</v>
+      </c>
+      <c r="N290" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P290" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>2</v>
+      </c>
+      <c r="C291" t="n">
+        <v>10</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F291" t="n">
+        <v>6</v>
+      </c>
+      <c r="G291" t="n">
+        <v>3</v>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Cezarro (IRE)</t>
+        </is>
+      </c>
+      <c r="I291" t="n">
+        <v>4</v>
+      </c>
+      <c r="J291" t="n">
+        <v>128</v>
+      </c>
+      <c r="K291" t="n">
+        <v>48</v>
+      </c>
+      <c r="L291" t="n">
+        <v>2</v>
+      </c>
+      <c r="M291" t="n">
+        <v>127.66</v>
+      </c>
+      <c r="N291" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P291" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>2</v>
+      </c>
+      <c r="C292" t="n">
+        <v>10</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F292" t="n">
+        <v>6</v>
+      </c>
+      <c r="G292" t="n">
+        <v>4</v>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>Duke Orsino</t>
+        </is>
+      </c>
+      <c r="I292" t="n">
+        <v>4</v>
+      </c>
+      <c r="J292" t="n">
+        <v>126</v>
+      </c>
+      <c r="K292" t="n">
+        <v>46</v>
+      </c>
+      <c r="L292" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="M292" t="n">
+        <v>127.66</v>
+      </c>
+      <c r="N292" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P292" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>2</v>
+      </c>
+      <c r="C293" t="n">
+        <v>10</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F293" t="n">
+        <v>6</v>
+      </c>
+      <c r="G293" t="n">
+        <v>5</v>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>Haveagobeau</t>
+        </is>
+      </c>
+      <c r="I293" t="n">
+        <v>7</v>
+      </c>
+      <c r="J293" t="n">
+        <v>132</v>
+      </c>
+      <c r="K293" t="n">
+        <v>52</v>
+      </c>
+      <c r="L293" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="M293" t="n">
+        <v>127.66</v>
+      </c>
+      <c r="N293" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P293" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>2</v>
+      </c>
+      <c r="C294" t="n">
+        <v>10</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F294" t="n">
+        <v>6</v>
+      </c>
+      <c r="G294" t="n">
+        <v>6</v>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>Crafter (IRE)</t>
+        </is>
+      </c>
+      <c r="I294" t="n">
+        <v>8</v>
+      </c>
+      <c r="J294" t="n">
+        <v>134</v>
+      </c>
+      <c r="K294" t="n">
+        <v>54</v>
+      </c>
+      <c r="L294" t="n">
+        <v>12.75</v>
+      </c>
+      <c r="M294" t="n">
+        <v>127.66</v>
+      </c>
+      <c r="N294" t="n">
+        <v>45</v>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P294" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>2</v>
+      </c>
+      <c r="C295" t="n">
+        <v>10</v>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F295" t="n">
+        <v>6</v>
+      </c>
+      <c r="G295" t="n">
+        <v>7</v>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Twilight Guest</t>
+        </is>
+      </c>
+      <c r="I295" t="n">
+        <v>6</v>
+      </c>
+      <c r="J295" t="n">
+        <v>130</v>
+      </c>
+      <c r="K295" t="n">
+        <v>50</v>
+      </c>
+      <c r="L295" t="n">
+        <v>14</v>
+      </c>
+      <c r="M295" t="n">
+        <v>127.66</v>
+      </c>
+      <c r="N295" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P295" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>2</v>
+      </c>
+      <c r="C296" t="n">
+        <v>10</v>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F296" t="n">
+        <v>6</v>
+      </c>
+      <c r="G296" t="n">
+        <v>8</v>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Stoneacre (IRE)</t>
+        </is>
+      </c>
+      <c r="I296" t="n">
+        <v>6</v>
+      </c>
+      <c r="J296" t="n">
+        <v>126</v>
+      </c>
+      <c r="K296" t="n">
+        <v>46</v>
+      </c>
+      <c r="L296" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="M296" t="n">
+        <v>127.66</v>
+      </c>
+      <c r="N296" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P296" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>3</v>
+      </c>
+      <c r="C297" t="n">
+        <v>9</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F297" t="n">
+        <v>4</v>
+      </c>
+      <c r="G297" t="n">
+        <v>1</v>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Sweet Reward (IRE)</t>
+        </is>
+      </c>
+      <c r="I297" t="n">
+        <v>9</v>
+      </c>
+      <c r="J297" t="n">
+        <v>135</v>
+      </c>
+      <c r="K297" t="n">
+        <v>85</v>
+      </c>
+      <c r="L297" t="inlineStr"/>
+      <c r="M297" t="n">
+        <v>113.19</v>
+      </c>
+      <c r="N297" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P297" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>3</v>
+      </c>
+      <c r="C298" t="n">
+        <v>9</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F298" t="n">
+        <v>4</v>
+      </c>
+      <c r="G298" t="n">
+        <v>2</v>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Footwork</t>
+        </is>
+      </c>
+      <c r="I298" t="n">
+        <v>4</v>
+      </c>
+      <c r="J298" t="n">
+        <v>136</v>
+      </c>
+      <c r="K298" t="n">
+        <v>86</v>
+      </c>
+      <c r="L298" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M298" t="n">
+        <v>113.19</v>
+      </c>
+      <c r="N298" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P298" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>3</v>
+      </c>
+      <c r="C299" t="n">
+        <v>9</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F299" t="n">
+        <v>4</v>
+      </c>
+      <c r="G299" t="n">
+        <v>3</v>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Epictetus (IRE)</t>
+        </is>
+      </c>
+      <c r="I299" t="n">
+        <v>6</v>
+      </c>
+      <c r="J299" t="n">
+        <v>131</v>
+      </c>
+      <c r="K299" t="n">
+        <v>81</v>
+      </c>
+      <c r="L299" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="M299" t="n">
+        <v>113.19</v>
+      </c>
+      <c r="N299" t="n">
+        <v>62</v>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P299" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>3</v>
+      </c>
+      <c r="C300" t="n">
+        <v>9</v>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F300" t="n">
+        <v>4</v>
+      </c>
+      <c r="G300" t="n">
+        <v>4</v>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>Quamby (IRE)</t>
+        </is>
+      </c>
+      <c r="I300" t="n">
+        <v>4</v>
+      </c>
+      <c r="J300" t="n">
+        <v>130</v>
+      </c>
+      <c r="K300" t="n">
+        <v>80</v>
+      </c>
+      <c r="L300" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="M300" t="n">
+        <v>113.19</v>
+      </c>
+      <c r="N300" t="n">
+        <v>55</v>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P300" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>3</v>
+      </c>
+      <c r="C301" t="n">
+        <v>9</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F301" t="n">
+        <v>4</v>
+      </c>
+      <c r="G301" t="n">
+        <v>5</v>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>Red Hat Eagle</t>
+        </is>
+      </c>
+      <c r="I301" t="n">
+        <v>6</v>
+      </c>
+      <c r="J301" t="n">
+        <v>127</v>
+      </c>
+      <c r="K301" t="n">
+        <v>77</v>
+      </c>
+      <c r="L301" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="M301" t="n">
+        <v>113.19</v>
+      </c>
+      <c r="N301" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P301" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B302" t="n">
+        <v>3</v>
+      </c>
+      <c r="C302" t="n">
+        <v>9</v>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F302" t="n">
+        <v>4</v>
+      </c>
+      <c r="G302" t="n">
+        <v>6</v>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Hitched (IRE)</t>
+        </is>
+      </c>
+      <c r="I302" t="n">
+        <v>6</v>
+      </c>
+      <c r="J302" t="n">
+        <v>128</v>
+      </c>
+      <c r="K302" t="n">
+        <v>78</v>
+      </c>
+      <c r="L302" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="M302" t="n">
+        <v>113.19</v>
+      </c>
+      <c r="N302" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P302" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B303" t="n">
+        <v>3</v>
+      </c>
+      <c r="C303" t="n">
+        <v>9</v>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F303" t="n">
+        <v>4</v>
+      </c>
+      <c r="G303" t="n">
+        <v>7</v>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Post Rider</t>
+        </is>
+      </c>
+      <c r="I303" t="n">
+        <v>5</v>
+      </c>
+      <c r="J303" t="n">
+        <v>128</v>
+      </c>
+      <c r="K303" t="n">
+        <v>78</v>
+      </c>
+      <c r="L303" t="n">
+        <v>11.15</v>
+      </c>
+      <c r="M303" t="n">
+        <v>113.19</v>
+      </c>
+      <c r="N303" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P303" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B304" t="n">
+        <v>4</v>
+      </c>
+      <c r="C304" t="n">
+        <v>4.986363636363636</v>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F304" t="n">
+        <v>4</v>
+      </c>
+      <c r="G304" t="n">
+        <v>1</v>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>Alta Regina (IRE)</t>
+        </is>
+      </c>
+      <c r="I304" t="n">
+        <v>2</v>
+      </c>
+      <c r="J304" t="n">
+        <v>128</v>
+      </c>
+      <c r="K304" t="n">
+        <v>0</v>
+      </c>
+      <c r="L304" t="inlineStr"/>
+      <c r="M304" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="N304" t="n">
+        <v>78.5</v>
+      </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P304" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B305" t="n">
+        <v>4</v>
+      </c>
+      <c r="C305" t="n">
+        <v>4.986363636363636</v>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F305" t="n">
+        <v>4</v>
+      </c>
+      <c r="G305" t="n">
+        <v>2</v>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Glamorize (IRE)</t>
+        </is>
+      </c>
+      <c r="I305" t="n">
+        <v>2</v>
+      </c>
+      <c r="J305" t="n">
+        <v>128</v>
+      </c>
+      <c r="K305" t="n">
+        <v>0</v>
+      </c>
+      <c r="L305" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="M305" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="N305" t="n">
+        <v>64</v>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P305" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>4</v>
+      </c>
+      <c r="C306" t="n">
+        <v>4.986363636363636</v>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F306" t="n">
+        <v>4</v>
+      </c>
+      <c r="G306" t="n">
+        <v>3</v>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>Roxa Love</t>
+        </is>
+      </c>
+      <c r="I306" t="n">
+        <v>2</v>
+      </c>
+      <c r="J306" t="n">
+        <v>128</v>
+      </c>
+      <c r="K306" t="n">
+        <v>0</v>
+      </c>
+      <c r="L306" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="M306" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="N306" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P306" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B307" t="n">
+        <v>4</v>
+      </c>
+      <c r="C307" t="n">
+        <v>4.986363636363636</v>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F307" t="n">
+        <v>4</v>
+      </c>
+      <c r="G307" t="n">
+        <v>4</v>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>Blue Sign</t>
+        </is>
+      </c>
+      <c r="I307" t="n">
+        <v>2</v>
+      </c>
+      <c r="J307" t="n">
+        <v>128</v>
+      </c>
+      <c r="K307" t="n">
+        <v>0</v>
+      </c>
+      <c r="L307" t="n">
+        <v>7.35</v>
+      </c>
+      <c r="M307" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="N307" t="n">
+        <v>52</v>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P307" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>4</v>
+      </c>
+      <c r="C308" t="n">
+        <v>4.986363636363636</v>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F308" t="n">
+        <v>4</v>
+      </c>
+      <c r="G308" t="n">
+        <v>5</v>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Matriarchal (IRE)</t>
+        </is>
+      </c>
+      <c r="I308" t="n">
+        <v>2</v>
+      </c>
+      <c r="J308" t="n">
+        <v>135</v>
+      </c>
+      <c r="K308" t="n">
+        <v>0</v>
+      </c>
+      <c r="L308" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="M308" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="N308" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P308" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B309" t="n">
+        <v>4</v>
+      </c>
+      <c r="C309" t="n">
+        <v>4.986363636363636</v>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F309" t="n">
+        <v>4</v>
+      </c>
+      <c r="G309" t="n">
+        <v>6</v>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Queencard (IRE)</t>
+        </is>
+      </c>
+      <c r="I309" t="n">
+        <v>2</v>
+      </c>
+      <c r="J309" t="n">
+        <v>128</v>
+      </c>
+      <c r="K309" t="n">
+        <v>0</v>
+      </c>
+      <c r="L309" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="M309" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="N309" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P309" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>4</v>
+      </c>
+      <c r="C310" t="n">
+        <v>4.986363636363636</v>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F310" t="n">
+        <v>4</v>
+      </c>
+      <c r="G310" t="n">
+        <v>7</v>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Targa (IRE)</t>
+        </is>
+      </c>
+      <c r="I310" t="n">
+        <v>2</v>
+      </c>
+      <c r="J310" t="n">
+        <v>128</v>
+      </c>
+      <c r="K310" t="n">
+        <v>0</v>
+      </c>
+      <c r="L310" t="n">
+        <v>8.65</v>
+      </c>
+      <c r="M310" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="N310" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P310" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>4</v>
+      </c>
+      <c r="C311" t="n">
+        <v>4.986363636363636</v>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F311" t="n">
+        <v>4</v>
+      </c>
+      <c r="G311" t="n">
+        <v>8</v>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>Charcoal Diva</t>
+        </is>
+      </c>
+      <c r="I311" t="n">
+        <v>2</v>
+      </c>
+      <c r="J311" t="n">
+        <v>128</v>
+      </c>
+      <c r="K311" t="n">
+        <v>0</v>
+      </c>
+      <c r="L311" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="M311" t="n">
+        <v>57.17</v>
+      </c>
+      <c r="N311" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="O311" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P311" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>5</v>
+      </c>
+      <c r="C312" t="n">
+        <v>7</v>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F312" t="n">
+        <v>4</v>
+      </c>
+      <c r="G312" t="n">
+        <v>0</v>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>Solar Maximus (IRE)</t>
+        </is>
+      </c>
+      <c r="I312" t="n">
+        <v>2</v>
+      </c>
+      <c r="J312" t="n">
+        <v>133</v>
+      </c>
+      <c r="K312" t="n">
+        <v>0</v>
+      </c>
+      <c r="L312" t="inlineStr"/>
+      <c r="M312" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="N312" t="inlineStr"/>
+      <c r="O312" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P312" t="n">
+        <v>-9</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>5</v>
+      </c>
+      <c r="C313" t="n">
+        <v>7</v>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F313" t="n">
+        <v>4</v>
+      </c>
+      <c r="G313" t="n">
+        <v>1</v>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>Sword Salute (USA)</t>
+        </is>
+      </c>
+      <c r="I313" t="n">
+        <v>2</v>
+      </c>
+      <c r="J313" t="n">
+        <v>130</v>
+      </c>
+      <c r="K313" t="n">
+        <v>0</v>
+      </c>
+      <c r="L313" t="inlineStr"/>
+      <c r="M313" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="N313" t="n">
+        <v>70.09999999999999</v>
+      </c>
+      <c r="O313" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P313" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>5</v>
+      </c>
+      <c r="C314" t="n">
+        <v>7</v>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F314" t="n">
+        <v>4</v>
+      </c>
+      <c r="G314" t="n">
+        <v>2</v>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>Gliding Martha (IRE)</t>
+        </is>
+      </c>
+      <c r="I314" t="n">
+        <v>2</v>
+      </c>
+      <c r="J314" t="n">
+        <v>128</v>
+      </c>
+      <c r="K314" t="n">
+        <v>0</v>
+      </c>
+      <c r="L314" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="M314" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="N314" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="O314" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P314" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B315" t="n">
+        <v>5</v>
+      </c>
+      <c r="C315" t="n">
+        <v>7</v>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F315" t="n">
+        <v>4</v>
+      </c>
+      <c r="G315" t="n">
+        <v>3</v>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>Able Tasman (IRE)</t>
+        </is>
+      </c>
+      <c r="I315" t="n">
+        <v>2</v>
+      </c>
+      <c r="J315" t="n">
+        <v>130</v>
+      </c>
+      <c r="K315" t="n">
+        <v>0</v>
+      </c>
+      <c r="L315" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="M315" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="N315" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="O315" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P315" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B316" t="n">
+        <v>5</v>
+      </c>
+      <c r="C316" t="n">
+        <v>7</v>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F316" t="n">
+        <v>4</v>
+      </c>
+      <c r="G316" t="n">
+        <v>4</v>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>Ariane Sky (IRE)</t>
+        </is>
+      </c>
+      <c r="I316" t="n">
+        <v>2</v>
+      </c>
+      <c r="J316" t="n">
+        <v>122</v>
+      </c>
+      <c r="K316" t="n">
+        <v>0</v>
+      </c>
+      <c r="L316" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="M316" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="N316" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="O316" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P316" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B317" t="n">
+        <v>5</v>
+      </c>
+      <c r="C317" t="n">
+        <v>7</v>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F317" t="n">
+        <v>4</v>
+      </c>
+      <c r="G317" t="n">
+        <v>5</v>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>Sakowin (IRE)</t>
+        </is>
+      </c>
+      <c r="I317" t="n">
+        <v>2</v>
+      </c>
+      <c r="J317" t="n">
+        <v>133</v>
+      </c>
+      <c r="K317" t="n">
+        <v>0</v>
+      </c>
+      <c r="L317" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="M317" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="N317" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="O317" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P317" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B318" t="n">
+        <v>5</v>
+      </c>
+      <c r="C318" t="n">
+        <v>7</v>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F318" t="n">
+        <v>4</v>
+      </c>
+      <c r="G318" t="n">
+        <v>6</v>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>Nakila Sun (GER)</t>
+        </is>
+      </c>
+      <c r="I318" t="n">
+        <v>2</v>
+      </c>
+      <c r="J318" t="n">
+        <v>127</v>
+      </c>
+      <c r="K318" t="n">
+        <v>0</v>
+      </c>
+      <c r="L318" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="M318" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="N318" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="O318" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P318" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B319" t="n">
+        <v>5</v>
+      </c>
+      <c r="C319" t="n">
+        <v>7</v>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F319" t="n">
+        <v>4</v>
+      </c>
+      <c r="G319" t="n">
+        <v>7</v>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>Wadima</t>
+        </is>
+      </c>
+      <c r="I319" t="n">
+        <v>2</v>
+      </c>
+      <c r="J319" t="n">
+        <v>125</v>
+      </c>
+      <c r="K319" t="n">
+        <v>0</v>
+      </c>
+      <c r="L319" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="M319" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="N319" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="O319" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P319" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B320" t="n">
+        <v>5</v>
+      </c>
+      <c r="C320" t="n">
+        <v>7</v>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F320" t="n">
+        <v>4</v>
+      </c>
+      <c r="G320" t="n">
+        <v>8</v>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>Pjs Corner</t>
+        </is>
+      </c>
+      <c r="I320" t="n">
+        <v>2</v>
+      </c>
+      <c r="J320" t="n">
+        <v>130</v>
+      </c>
+      <c r="K320" t="n">
+        <v>0</v>
+      </c>
+      <c r="L320" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="M320" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="N320" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="O320" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="P320" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B321" t="n">
+        <v>6</v>
+      </c>
+      <c r="C321" t="n">
+        <v>7.613636363636363</v>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F321" t="n">
+        <v>5</v>
+      </c>
+      <c r="G321" t="n">
+        <v>1</v>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>Get Outta Here (FR)</t>
+        </is>
+      </c>
+      <c r="I321" t="n">
+        <v>3</v>
+      </c>
+      <c r="J321" t="n">
+        <v>130</v>
+      </c>
+      <c r="K321" t="n">
+        <v>70</v>
+      </c>
+      <c r="L321" t="inlineStr"/>
+      <c r="M321" t="n">
+        <v>90.86</v>
+      </c>
+      <c r="N321" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="O321" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P321" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B322" t="n">
+        <v>6</v>
+      </c>
+      <c r="C322" t="n">
+        <v>7.613636363636363</v>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F322" t="n">
+        <v>5</v>
+      </c>
+      <c r="G322" t="n">
+        <v>2</v>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>Vidmiyr (IRE)</t>
+        </is>
+      </c>
+      <c r="I322" t="n">
+        <v>3</v>
+      </c>
+      <c r="J322" t="n">
+        <v>135</v>
+      </c>
+      <c r="K322" t="n">
+        <v>75</v>
+      </c>
+      <c r="L322" t="n">
+        <v>1</v>
+      </c>
+      <c r="M322" t="n">
+        <v>90.86</v>
+      </c>
+      <c r="N322" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="O322" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P322" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B323" t="n">
+        <v>6</v>
+      </c>
+      <c r="C323" t="n">
+        <v>7.613636363636363</v>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F323" t="n">
+        <v>5</v>
+      </c>
+      <c r="G323" t="n">
+        <v>3</v>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>Raging Raj (IRE)</t>
+        </is>
+      </c>
+      <c r="I323" t="n">
+        <v>3</v>
+      </c>
+      <c r="J323" t="n">
+        <v>134</v>
+      </c>
+      <c r="K323" t="n">
+        <v>74</v>
+      </c>
+      <c r="L323" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M323" t="n">
+        <v>90.86</v>
+      </c>
+      <c r="N323" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="O323" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P323" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B324" t="n">
+        <v>6</v>
+      </c>
+      <c r="C324" t="n">
+        <v>7.613636363636363</v>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F324" t="n">
+        <v>5</v>
+      </c>
+      <c r="G324" t="n">
+        <v>4</v>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>Velvet Rhythm</t>
+        </is>
+      </c>
+      <c r="I324" t="n">
+        <v>3</v>
+      </c>
+      <c r="J324" t="n">
+        <v>128</v>
+      </c>
+      <c r="K324" t="n">
+        <v>68</v>
+      </c>
+      <c r="L324" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="M324" t="n">
+        <v>90.86</v>
+      </c>
+      <c r="N324" t="n">
+        <v>60</v>
+      </c>
+      <c r="O324" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P324" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B325" t="n">
+        <v>6</v>
+      </c>
+      <c r="C325" t="n">
+        <v>7.613636363636363</v>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F325" t="n">
+        <v>5</v>
+      </c>
+      <c r="G325" t="n">
+        <v>5</v>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>Accademia</t>
+        </is>
+      </c>
+      <c r="I325" t="n">
+        <v>3</v>
+      </c>
+      <c r="J325" t="n">
+        <v>127</v>
+      </c>
+      <c r="K325" t="n">
+        <v>67</v>
+      </c>
+      <c r="L325" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="M325" t="n">
+        <v>90.86</v>
+      </c>
+      <c r="N325" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="O325" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P325" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B326" t="n">
+        <v>6</v>
+      </c>
+      <c r="C326" t="n">
+        <v>7.613636363636363</v>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F326" t="n">
+        <v>5</v>
+      </c>
+      <c r="G326" t="n">
+        <v>6</v>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>Berkshire Boom (IRE)</t>
+        </is>
+      </c>
+      <c r="I326" t="n">
+        <v>3</v>
+      </c>
+      <c r="J326" t="n">
+        <v>133</v>
+      </c>
+      <c r="K326" t="n">
+        <v>73</v>
+      </c>
+      <c r="L326" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="M326" t="n">
+        <v>90.86</v>
+      </c>
+      <c r="N326" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="O326" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P326" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B327" t="n">
+        <v>7</v>
+      </c>
+      <c r="C327" t="n">
+        <v>6</v>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F327" t="n">
+        <v>5</v>
+      </c>
+      <c r="G327" t="n">
+        <v>0</v>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>Woolridge</t>
+        </is>
+      </c>
+      <c r="I327" t="n">
+        <v>4</v>
+      </c>
+      <c r="J327" t="n">
+        <v>125</v>
+      </c>
+      <c r="K327" t="n">
+        <v>62</v>
+      </c>
+      <c r="L327" t="inlineStr"/>
+      <c r="M327" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="N327" t="inlineStr"/>
+      <c r="O327" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P327" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B328" t="n">
+        <v>7</v>
+      </c>
+      <c r="C328" t="n">
+        <v>6</v>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F328" t="n">
+        <v>5</v>
+      </c>
+      <c r="G328" t="n">
+        <v>1</v>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>Twilight Jet (IRE)</t>
+        </is>
+      </c>
+      <c r="I328" t="n">
+        <v>7</v>
+      </c>
+      <c r="J328" t="n">
+        <v>140</v>
+      </c>
+      <c r="K328" t="n">
+        <v>77</v>
+      </c>
+      <c r="L328" t="inlineStr"/>
+      <c r="M328" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="N328" t="n">
+        <v>75.3</v>
+      </c>
+      <c r="O328" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P328" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B329" t="n">
+        <v>7</v>
+      </c>
+      <c r="C329" t="n">
+        <v>6</v>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F329" t="n">
+        <v>5</v>
+      </c>
+      <c r="G329" t="n">
+        <v>2</v>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>Invincible Speed (IRE)</t>
+        </is>
+      </c>
+      <c r="I329" t="n">
+        <v>5</v>
+      </c>
+      <c r="J329" t="n">
+        <v>134</v>
+      </c>
+      <c r="K329" t="n">
+        <v>71</v>
+      </c>
+      <c r="L329" t="n">
+        <v>4</v>
+      </c>
+      <c r="M329" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="N329" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="O329" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P329" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B330" t="n">
+        <v>7</v>
+      </c>
+      <c r="C330" t="n">
+        <v>6</v>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F330" t="n">
+        <v>5</v>
+      </c>
+      <c r="G330" t="n">
+        <v>3</v>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>The Bitter Moose (IRE)</t>
+        </is>
+      </c>
+      <c r="I330" t="n">
+        <v>5</v>
+      </c>
+      <c r="J330" t="n">
+        <v>134</v>
+      </c>
+      <c r="K330" t="n">
+        <v>71</v>
+      </c>
+      <c r="L330" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="M330" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="N330" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="O330" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P330" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B331" t="n">
+        <v>7</v>
+      </c>
+      <c r="C331" t="n">
+        <v>6</v>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F331" t="n">
+        <v>5</v>
+      </c>
+      <c r="G331" t="n">
+        <v>4</v>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>Mission Command (IRE)</t>
+        </is>
+      </c>
+      <c r="I331" t="n">
+        <v>4</v>
+      </c>
+      <c r="J331" t="n">
+        <v>136</v>
+      </c>
+      <c r="K331" t="n">
+        <v>73</v>
+      </c>
+      <c r="L331" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="M331" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="N331" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="O331" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P331" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>LINGFIELD PARK</t>
+        </is>
+      </c>
+      <c r="B332" t="n">
+        <v>7</v>
+      </c>
+      <c r="C332" t="n">
+        <v>6</v>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Good To Firm</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Turf</t>
+        </is>
+      </c>
+      <c r="F332" t="n">
+        <v>5</v>
+      </c>
+      <c r="G332" t="n">
+        <v>5</v>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>Lahina Bay (IRE)</t>
+        </is>
+      </c>
+      <c r="I332" t="n">
+        <v>6</v>
+      </c>
+      <c r="J332" t="n">
+        <v>123</v>
+      </c>
+      <c r="K332" t="n">
+        <v>60</v>
+      </c>
+      <c r="L332" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="M332" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="N332" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="O332" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P332" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>